<commit_message>
Remove cell comments, add CSV version
</commit_message>
<xml_diff>
--- a/walls_dataset.xlsx
+++ b/walls_dataset.xlsx
@@ -20,2219 +20,6 @@
     </ext>
   </extLst>
 </workbook>
-</file>
-
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Author</author>
-  </authors>
-  <commentList>
-    <comment ref="A5" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Almost every information about these two specimens was erroneous. Many corrections were applied</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A292" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGs
-Yazar    (2020-07-05 18:02:42)
-Data from University of Patras incompatible with the data from the paper. No other reference was found for controlling purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A294" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKE
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curves are not proper for the project purposes.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A313" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJk
-Yazar    (2020-07-05 18:02:42)
-Axial Load varies throughout the test.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B42" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRIE
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curve is missing</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B43" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRLc
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curve is missing</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B44" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNM
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curve is missing</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B59" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRH8
-Yazar    (2020-07-05 18:02:42)
-Attempt for digitising this specimen was unsuccessful</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B63" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRMI
-Yazar    (2020-07-05 18:02:42)
-Not proper for the research purposes because of varying axial load throughout the test</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B64" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRMs
-Yazar    (2020-07-05 18:02:42)
-Not proper for the research purposes because of varying axial load throughout the test</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B88" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGA
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B89" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNo
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B90" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKM
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B91" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRMg
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B92" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGI
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B93" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROU
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B94" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRM8
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B109" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRI0
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B110" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGk
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B111" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRIs
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curves for specimens NO.1 to NO.8 not available
-only the backbone curves are available.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B113" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRF0
-Yazar    (2020-07-05 18:02:42)
-drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B118" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRFs
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curves for specimens NO.1 to NO.8 not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B122" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGM
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B123" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRLk
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B125" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROs
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B135" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROo
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B136" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKY
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B137" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRH4
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B139" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRN8
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B145" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROw
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B174" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B175" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B177" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B178" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B180" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B181" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B182" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B183" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B185" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B186" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B188" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B191" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B192" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ0
-Yazar    (2020-07-05 18:02:42)
-The hysteretic curve is not appropriate for the research purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B203" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNc
-Yazar    (2020-07-05 18:02:42)
-NOT PROPER for 1% drift ratio studies but, PROPER for cumulative energy studies</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B204" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJE
-Yazar    (2020-07-05 18:02:42)
-NOT PROPER for 1% drift ratio studies but, PROPER for cumulative energy studies</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B207" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRMM
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B208" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRMM
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B209" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHc
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B225" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHg
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B226" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRLY
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B227" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRFk
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B228" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNk
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B229" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Hysteretis curve not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B230" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRLQ
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B237" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRFw
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B238" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHs
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B239" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJo
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B240" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRME
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B248" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRIA
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B249" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRM4
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B250" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRLo
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B252" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Specimens recognised with "H" are subjected to bilateral out of plane loading and probably should not be used in the current study where specimens subjected to uni-lateral loadings are of interest</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B253" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Specimens recognised with "H" are subjected to bilateral out of plane loading and probably should not be used in the current study where specimens subjected to uni-lateral loadings are of interest</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B254" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Specimens recognised with "H" are subjected to bilateral out of plane loading and probably should not be used in the current study where specimens subjected to uni-lateral loadings are of interest</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B255" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Specimens recognised with "H" are subjected to bilateral out of plane loading and probably should not be used in the current study where specimens subjected to uni-lateral loadings are of interest</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B256" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRO8
-Yazar    (2020-07-05 18:02:42)
-Specimens T2-S1 and T2-S2 (at the bottom of the inventory) differed in
-terms of anchorage conditions of horizontal web reinforcement:
-Specimen T2-S1 had U-cap hooks at the ends of the horizontal web bars,
-while specimen T2-S2, as well as all other specimens, had 180° hooks at
-the end of the horizontal bars. So, T2-S1 specimen is not used.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B268" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKg
-Yazar    (2020-07-05 18:02:42)
-Yazar
-Hysteretic curve only available for the push side (identified as not appropriate for the project purposes)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B282" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJc
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B283" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROM
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B286" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROQ
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B287" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNQ
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B288" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHM
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B289" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKU
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B290" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKc
-Yazar    (2020-07-05 18:02:42)
-1% Drift Ratio'ya ulaşamamıştır.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B291" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRL4
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B324" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHU
-Yazar    (2020-07-05 18:02:42)
-Two 10 &amp; 7 storey frames with shear walls were tested. Not appropriate for the project purposes</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B326" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHw
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B327" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJQ
-Yazar    (2020-07-05 18:02:42)
-%1 Drift Ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B328" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHE
-Yazar    (2020-07-05 18:02:42)
-Specimens T2-S1 and T2-S2 differed in
-terms of anchorage conditions of horizontal web reinforcement:
-Specimen T2-S1 had U-cap hooks at the ends of the horizontal web bars,
-while specimen T2-S2, as well as all other specimens, had 180° hooks at
-the end of the horizontal bars</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B329" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGw
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B330" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJA
-Yazar    (2020-07-05 18:02:42)
-%1 drift ratio criterion is not fulfilled.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B331" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRMw
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curve not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B332" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHI
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curve and backbone curve not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B333" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNY
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curve and backbone curve not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B334" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRFo
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curves for specimens W48M6, W48M4, W72M8, W96M8 not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B335" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHA
-Yazar    (2020-07-05 18:02:42)
-Hysteretic curves for specimens W48M6, W48M4, W72M8, W96M8 not available</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGY
-Siamak    (2020-07-05 18:02:42)
-1:Rectengular
-2:Barbell
-3:Flanged</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRI8
-Yazar    (2020-07-05 18:02:42)
-Failure Type:
-0:Not failed
-1: Shear
-2: Mix
-3: Flexural</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I232" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Sliding shear (pp. 23)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJI
-Yazar    (2020-07-05 18:02:42)
-Curvature Type:
-1: Single curvature
-2: Double curvature</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M81" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M82" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M83" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M84" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M85" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M86" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M87" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Cited from Sengupta &amp; Li (2014) due to insufficient information in the main reference (Hidalgo et al, 2002)</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M237" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M238" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M239" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M240" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M241" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M242" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M243" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O214" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Was modified as a result of change in legs No.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O217" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Was modified as a result of change in legs No.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O237" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O238" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O239" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O240" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O241" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O242" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O243" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O251" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel ratio was rectified as a result of correcting leg numbers</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O252" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel ratio was rectified as a result of correcting leg numbers</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O254" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel ratio was rectified as a result of correcting leg numbers</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O255" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel ratio was rectified as a result of correcting leg numbers</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O269" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Slightly changed as s was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O270" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Slightly changed as s was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O271" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Slightly changed as s was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O272" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Slightly changed as s was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O273" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Slightly changed as s was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P237" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P238" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P239" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P240" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P241" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P242" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P243" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R6" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-it changed from %0.74 to %0.60</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R211" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Corrected from 0.54 to 0.66</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R212" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Corrected from 0.54 to 0.66</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R213" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Corrected from 0.54 to 0.66</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R214" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Corrected from 0.88 to 0.52</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R220" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-ρl was rectified as a result of correcting distance between Long. Rebars.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R235" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Boundary region is assumed not to exist. Consequently, long. steel ratio in the web region is modified.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R236" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-Boundary region is assumed not to exist. Consequently, long. steel ratio in the web region is modified.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R237" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R238" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R239" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R240" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R241" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R242" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R243" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Author:
-steel rario changed slightly as Dnom was modified</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U1" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRKA
-Yazar    (2020-07-05 18:02:42)
-1: Force-Control
-2:Displacement-Control
-3-Force control before displacement control
-4-Displacement-control before force-control
-İncremental İnformation :
-0-Constant
-1-One cycle incremental
-2-Two cycle incremental
-Final Code Example:
-10-Force Control Constant
-11-Force Control one cycle incremental (1 çevrimde artımlı yükleme çeşidi)
-22-Displacement-Control two cycle incremental (2 çevrimde bir artımlı yükleme çeşidi)
-3 ve 4 özel yükleme çeşitleri olduğundan bu protocola sahip olanlar ayrıca incelenmelidir!</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U137" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRJ8
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U138" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRNE
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U139" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRH0
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U140" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRLg
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U141" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLROY
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U142" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRGE
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U143" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRG4
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U144" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">======
-ID#AAAAJviLRHY
-Yazar    (2020-07-05 18:02:42)
-1 cycle loading is applied to the first step only.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -34410,6 +32197,5 @@
     <oddFooter/>
   </headerFooter>
   <drawing r:id="rId2"/>
-  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>